<commit_message>
chore: update news radar report 2026-07-30
</commit_message>
<xml_diff>
--- a/docs/data/rxbenefits_intel_hub_report_2026-07-30.xlsx
+++ b/docs/data/rxbenefits_intel_hub_report_2026-07-30.xlsx
@@ -446,54 +446,54 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Employers Face Growing Cancer Care Gaps and Surging Costs Amid Lagging Precision Medicine Adoption</t>
+          <t>Cigna Elevates Annual Profit Outlook Driven By Health Services Growth</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>A new study reveals that self-funded employers are confronting a significant "cancer attention gap" as treatment costs surge and access to advanced precision care lags behind. This matters because cancer remains one of the largest drivers of catastrophic claims in employer-sponsored health plans, threatening corporate healthcare budgets. The key business implication is an urgent need for pharmacy benefits and plan management strategies that better integrate oncology navigation, manage specialty drug costs, and optimize targeted therapies to control employer spending.</t>
+          <t>Cigna has raised its full-year profit forecast, fueled by strong performance within its health services division, Evernorth, which manages pharmacy benefits and specialty care. This growth highlights the increasing financial power and market demand for integrated pharmacy and healthcare navigation solutions. For self-funded employers and the broader benefits market, this trend underscores the shifting dynamics of PBM-driven services and healthcare cost management strategies.</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Yahoo Finance</t>
+          <t>The Mighty 790 KFGO</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Wed, 29 Jul 2026 13:00:00 GMT</t>
+          <t>Thu, 30 Jul 2026 10:20:21 GMT</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxPUDBFOXctOFNSanJmakZrVV92RHNPaEZYLUthTUNNNDA5NGI4dWV4QlJ1cGE2YlFfRkp4TXMxeTBXaWZpdTh4Wk1pMXNpTWJQNWdEcTc0REppTm0yc2RJZFgtd011UDIwa1B2WElZSE5jMEVQQUVVWF9HS0tkZGo4Q2NCU2xPSlV6NEtEMUZMaVVvVm1RTmpFX2sxX2xKZw?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMiogFBVV95cUxQSXhVLUpNaEtSYkY1ajc3VWRmY0txVHJhVHZ0OGlZLWVvZFlrSGg2VFRNWXNER0ZkR2pmSXFZOGNzYlNxQk1vTXZnM0R2SGhKeUhJMWNEbU93NExhZ2drcERHZGlLaHJOR3N0ZlBVQVZLZXN1YTlPVHA1N1c1YzNCUHNub0thUlFZRGlhQ0xET01LbU9rVEhLV0dEdVdPdjNCRnc?oc=5</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Wellcentra and LaborForce Media Partner to Combat Plan Sponsor Drug Costs</t>
+          <t>New Study Reveals Growing Cancer Care Gap and Surging Costs for Self-Funded Employers</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Wellcentra and LaborForce Media have announced a strategic partnership aimed at helping self-funded plan sponsors navigate and mitigate escalating prescription drug expenditures. This alliance matters because rising specialty and brand-name drug prices continue to strain employer-sponsored health plans, demanding innovative cost-containment strategies. For business operations, this collaboration provides plan sponsors with enhanced educational resources and advisory tools to optimize pharmacy benefit management, improve plan performance, and better control long-term healthcare liabilities.</t>
+          <t>A recent study highlights that self-funded employers are facing a significant "cancer attention gap" as treatment costs surge and access to precision care lags behind. This matters because cancer remains one of the largest drivers of employer-sponsored health plan expenditures, putting immense pressure on corporate healthcare budgets. The key business implication is that pharmacy and benefits managers must implement more targeted oncology navigation and precision medicine strategies to control costs while improving employee health outcomes.</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>The National Law Review</t>
+          <t>Yahoo Finance</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Wed, 29 Jul 2026 10:13:06 GMT</t>
+          <t>Wed, 29 Jul 2026 13:00:00 GMT</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://news.google.com/rss/articles/CBMiswFBVV95cUxQekRSelBrZGNRU2RqYWdjbE01Ujg3LXpfY0VVUzdXNzctbFg0N0FTNU96c3V4aFdLWFFsX1ZSd253UFRBR0tpRkg3MWNLSmI3Tkk2bEsxWnlOSHg0aVJwR1RKcEt3TmNYdl85dFRyMTFXcmNjakRBMnRLUGJMM2RoS1FOUDV5WHlJUFBQdkV4c2FTSWgzRXNibUduNmJnbzhqNWo0d0xEamRUWjIySE4yb2RwTQ?oc=5</t>
+          <t>https://news.google.com/rss/articles/CBMingFBVV95cUxPUDBFOXctOFNSanJmakZrVV92RHNPaEZYLUthTUNNNDA5NGI4dWV4QlJ1cGE2YlFfRkp4TXMxeTBXaWZpdTh4Wk1pMXNpTWJQNWdEcTc0REppTm0yc2RJZFgtd011UDIwa1B2WElZSE5jMEVQQUVVWF9HS0tkZGo4Q2NCU2xPSlV6NEtEMUZMaVVvVm1RTmpFX2sxX2xKZw?oc=5</t>
         </is>
       </c>
     </row>

</xml_diff>